<commit_message>
Doctor jobs update - 29 Jun 2026 18:08 AEST
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -439,7 +439,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -547,7 +547,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="51" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1120,7 +1120,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -1798,7 +1798,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -2301,7 +2301,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -2409,7 +2409,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -3381,7 +3381,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -3415,8 +3414,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3444,7 +3441,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -3478,8 +3474,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3507,7 +3501,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -3541,8 +3534,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3570,7 +3561,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -3604,8 +3594,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3619,7 +3607,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -3727,7 +3715,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -3834,8 +3822,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
@@ -4939,6 +4927,534 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SmartJobs_QLD</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Jobs_NT</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Careers_VIC</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Monash_Health</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>23</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Western_Health</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>8</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>WA_Health</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Peninsula_Health</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>The_Womens</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Grampians_Health</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>8</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Eastern_Health</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>10</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>RCH</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>7</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>RANZCOG</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>RACP</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>21</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>JobRadars</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>403 Client Error: Forbidden for url: https://australia.jobradars.com/jobs?q=registrar+medical</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PageUp</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>pageup</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Mercy_Workday</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4951,7 +5467,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -6489,7 +7005,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -8399,7 +8915,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -8433,8 +8948,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10742,7 +11255,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -10776,8 +11288,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr"/>
-      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10805,7 +11315,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -10839,8 +11348,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10868,7 +11375,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -10902,8 +11408,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr"/>
-      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -10931,7 +11435,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -10965,8 +11468,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr"/>
-      <c r="O78" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17354,7 +17855,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -17462,7 +17963,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -18850,7 +19351,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -19372,7 +19873,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -19406,8 +19906,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19421,7 +19919,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -19529,7 +20027,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -19637,7 +20135,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
@@ -19745,7 +20243,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>

</xml_diff>

<commit_message>
Doctor jobs update - 29 Jun 2026 20:26 AEST
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -1191,7 +1191,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -1225,8 +1224,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1239,7 +1236,6 @@
           <t>ICU</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>Grampians Health</t>
@@ -1255,7 +1251,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -1289,8 +1284,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1323,7 +1316,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -1357,8 +1349,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1371,7 +1361,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Grampians Health</t>
@@ -1387,7 +1376,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -1421,8 +1409,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1455,7 +1441,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -1489,8 +1474,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1498,7 +1481,6 @@
           <t>International Job Seekers</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Intern</t>
@@ -1519,7 +1501,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -1553,8 +1534,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2301,7 +2280,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>Eastern Health</t>
@@ -2317,7 +2295,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -2351,8 +2328,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2360,7 +2335,6 @@
           <t>2027 Upper Gastro Intestinal Research Fellow</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Fellow</t>
@@ -2381,7 +2355,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -2415,8 +2388,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2585,11 +2556,11 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. Michael O'Brien</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -2769,7 +2740,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -2894,7 +2865,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -2954,7 +2925,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -4376,7 +4347,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4410,7 +4380,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -4448,7 +4417,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4482,7 +4450,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -4520,7 +4487,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4554,7 +4520,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -4592,7 +4557,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4626,7 +4590,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -4644,7 +4607,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -4660,7 +4622,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4694,8 +4655,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4708,7 +4667,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -4724,7 +4682,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4758,8 +4715,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4772,7 +4727,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -4788,7 +4742,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4822,8 +4775,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4836,7 +4787,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -4852,7 +4802,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4886,8 +4835,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4900,7 +4847,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -4916,7 +4862,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -4950,8 +4895,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4964,7 +4907,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -4980,7 +4922,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5014,8 +4955,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5048,7 +4987,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5082,8 +5020,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5116,7 +5052,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5150,8 +5085,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5184,7 +5117,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5218,8 +5150,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5252,7 +5182,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5286,8 +5215,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5320,7 +5247,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5354,8 +5280,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5388,7 +5312,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5422,8 +5345,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5456,7 +5377,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5490,8 +5410,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -5504,7 +5422,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -5520,7 +5437,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5554,8 +5470,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5563,7 +5477,6 @@
           <t>International Grants</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>Intern</t>
@@ -5584,7 +5497,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5618,8 +5530,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5627,7 +5537,6 @@
           <t>Prizes, grants, scholarships and fellowships</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>Fellow</t>
@@ -5648,7 +5557,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -5682,8 +5590,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5924,7 +5830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7554,6 +7460,534 @@
       <c r="G49" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SmartJobs_QLD</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Jobs_NT</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Careers_VIC</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Monash_Health</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>23</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Western_Health</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>12</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>WA_Health</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Peninsula_Health</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>The_Womens</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Grampians_Health</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>14</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Eastern_Health</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>12</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>RCH</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>7</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>RANZCOG</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>RACP</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>41</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>JobRadars</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>PageUp</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>pageup</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>29-06-2026</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Mercy_Workday</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>workday</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>auto-disabled</t>
         </is>
       </c>
     </row>
@@ -7666,12 +8100,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Grampians_Health</t>
+          <t>RCH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Registrar - General Medicine Advanced Trainee</t>
+          <t>2027 Senior Registrar General Medicine</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -7681,12 +8115,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Senior Registrar</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Grampians Health</t>
+          <t>Royal Children's Hospital</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -7701,11 +8135,11 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Registrar-General-Medicine-Advanced-Trainee-VIC-3350/1362283766/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -7726,32 +8160,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Michael O'Brien</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Western_Health</t>
+          <t>Grampians_Health</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2027 Emergency Medicine Medical Officer</t>
+          <t>Registrar - General Medicine Advanced Trainee</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Emergency Medicine</t>
+          <t>General Medicine</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Medical Officer</t>
+          <t>Registrar</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Western Health</t>
+          <t>Grampians Health</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -7766,11 +8200,11 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://careers.wh.org.au/job/2027-Emergency-Medicine-Medical-Officer/1361118766/</t>
+          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Registrar-General-Medicine-Advanced-Trainee-VIC-3350/1362283766/</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -7791,7 +8225,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dr. Priya Sharma</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -7801,17 +8235,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>General Practitioner - Custodial Health</t>
+          <t>2027 Emergency Medicine Medical Officer</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>General Practitioner (GP)</t>
+          <t>Emergency Medicine</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>General Practitioner (GP)</t>
+          <t>Medical Officer</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -7831,11 +8265,11 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://careers.wh.org.au/job/General-Practitioner-Custodial-Health/1359743566/</t>
+          <t>https://careers.wh.org.au/job/2027-Emergency-Medicine-Medical-Officer/1361118766/</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -7848,11 +8282,7 @@
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>High Match</t>
-        </is>
-      </c>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -7860,47 +8290,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Priya Sharma</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>RACP</t>
+          <t>Western_Health</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Adult Internal Medicine</t>
+          <t>General Practitioner - Custodial Health</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Paediatrics</t>
+          <t>General Practitioner (GP)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>General Practitioner (GP)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>RACP Member Hospital (AU)</t>
+          <t>Western Health</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>nt</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/basic-training/adult-internal-medicine</t>
+          <t>https://careers.wh.org.au/job/General-Practitioner-Custodial-Health/1359743566/</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -7917,7 +8347,11 @@
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>High Match</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -7935,7 +8369,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Paediatrics &amp; Child Health</t>
+          <t>Adult Internal Medicine</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -7943,7 +8377,11 @@
           <t>Paediatrics</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -7961,7 +8399,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/basic-training/paediatrics-child-health</t>
+          <t>https://www.racp.edu.au/trainees/basic-training/adult-internal-medicine</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -7996,7 +8434,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Addiction Medicine</t>
+          <t>Paediatrics &amp; Child Health</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -8022,7 +8460,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/addiction-medicine</t>
+          <t>https://www.racp.edu.au/trainees/basic-training/paediatrics-child-health</t>
         </is>
       </c>
       <c r="K7" t="n">
@@ -8057,7 +8495,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Adolescent and Young Adult Medicine</t>
+          <t>Addiction Medicine</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -8083,7 +8521,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/adolescent-and-young-adult-medicine</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/addiction-medicine</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -8118,19 +8556,15 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Post-Fellowship training</t>
+          <t>Adolescent and Young Adult Medicine</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Internal Medicine</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Fellow</t>
-        </is>
-      </c>
+          <t>Paediatrics</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -8148,7 +8582,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/multi-specialty-training-options/post-fellowship-training</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/adolescent-and-young-adult-medicine</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -8165,11 +8599,7 @@
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>High Match</t>
-        </is>
-      </c>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8187,7 +8617,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Post-Fellowship training</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -8217,7 +8647,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/cardiology</t>
+          <t>https://www.racp.edu.au/trainees/multi-specialty-training-options/post-fellowship-training</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -8256,7 +8686,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New curricula</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -8286,7 +8716,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/new-curricula</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/cardiology</t>
         </is>
       </c>
       <c r="K11" t="n">
@@ -8325,7 +8755,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Advanced Training - New Curricula</t>
+          <t>New curricula</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8355,7 +8785,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/recognition-of-prior-learning/advanced-training-new-curricula</t>
+          <t>https://www.racp.edu.au/trainees/new-curricula</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -8384,51 +8814,51 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dr. Priya Sharma</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Monash_Health</t>
+          <t>RACP</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2027 Obstetric &amp; Gynaecology - Senior Registrar</t>
+          <t>Advanced Training - New Curricula</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Gynaecology</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Senior Registrar</t>
+          <t>Fellow</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Monash Health</t>
+          <t>RACP Member Hospital (AU)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>nt</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://careers.monashhealth.org/job/Clayton-2027-Obstetric-&amp;-Gynaecology-Senior-Registrar-VIC-3168/1362522866/</t>
+          <t>https://www.racp.edu.au/trainees/recognition-of-prior-learning/advanced-training-new-curricula</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -8441,7 +8871,11 @@
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>High Match</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -8454,17 +8888,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eastern_Health</t>
+          <t>Monash_Health</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2027 Senior Registrar - Obstetrics &amp; Gynaecology</t>
+          <t>2027 Obstetric &amp; Gynaecology - Senior Registrar</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Obstetrics</t>
+          <t>Gynaecology</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -8474,7 +8908,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Eastern Health</t>
+          <t>Monash Health</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -8489,7 +8923,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://careers.easternhealth.org.au/job/Eastern-Health-2027-Senior-Registrar-Obstetrics-&amp;-Gynaecology-VIC-3128/1362270666/</t>
+          <t>https://careers.monashhealth.org/job/Clayton-2027-Obstetric-&amp;-Gynaecology-Senior-Registrar-VIC-3168/1362522866/</t>
         </is>
       </c>
       <c r="K14" t="n">
@@ -8514,20 +8948,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Priya Sharma</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Monash_Health</t>
+          <t>Eastern_Health</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2027 Intensive Care Registrar and Senior Registrars  - MMC &amp; VHH</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>2027 Senior Registrar - Obstetrics &amp; Gynaecology</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Obstetrics</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>Senior Registrar</t>
@@ -8535,7 +8973,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Monash Health</t>
+          <t>Eastern Health</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -8550,15 +8988,15 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://careers.monashhealth.org/job/Clayton-2027-Intensive-Care-Registrar-and-Senior-Registrars-MMC-&amp;-VHH-VIC-3168/1360917466/</t>
+          <t>https://careers.easternhealth.org.au/job/Eastern-Health-2027-Senior-Registrar-Obstetrics-&amp;-Gynaecology-VIC-3128/1362270666/</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Good Match</t>
+          <t>High Match</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -8575,32 +9013,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dr. Priya Sharma</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Western_Health</t>
+          <t>Monash_Health</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2027 Senior Obstetric &amp; Gynaecology Registrars</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Gynaecology</t>
-        </is>
-      </c>
+          <t>2027 Intensive Care Registrar and Senior Registrars  - MMC &amp; VHH</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Senior Registrar</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Western Health</t>
+          <t>Monash Health</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -8615,7 +9049,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://careers.wh.org.au/job/2027-Senior-Obstetric-&amp;-Gynaecology-Registrars/1362020866/</t>
+          <t>https://careers.monashhealth.org/job/Clayton-2027-Intensive-Care-Registrar-and-Senior-Registrars-MMC-&amp;-VHH-VIC-3168/1360917466/</t>
         </is>
       </c>
       <c r="K16" t="n">
@@ -8645,17 +9079,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Grampians_Health</t>
+          <t>Western_Health</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Registrar - Obstetrics &amp; Gynaecology Unaccredited</t>
+          <t>2027 Senior Obstetric &amp; Gynaecology Registrars</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Obstetrics</t>
+          <t>Gynaecology</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -8665,7 +9099,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Grampians Health</t>
+          <t>Western Health</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -8680,7 +9114,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Registrar-Obstetrics-&amp;-Gynaecology-Unaccredited-VIC-3350/1357598066/</t>
+          <t>https://careers.wh.org.au/job/2027-Senior-Obstetric-&amp;-Gynaecology-Registrars/1362020866/</t>
         </is>
       </c>
       <c r="K17" t="n">
@@ -8715,7 +9149,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Obstetrics &amp; Gynaecology Registrar (Accredited)</t>
+          <t>Registrar - Obstetrics &amp; Gynaecology Unaccredited</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -8745,7 +9179,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Obstetrics-&amp;-Gynaecology-Registrar-%28Accredited%29-VIC-3350/1362508966/</t>
+          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Registrar-Obstetrics-&amp;-Gynaecology-Unaccredited-VIC-3350/1357598066/</t>
         </is>
       </c>
       <c r="K18" t="n">
@@ -8770,32 +9204,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. Priya Sharma</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>RCH</t>
+          <t>Grampians_Health</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2027 Senior Registrar General Medicine</t>
+          <t>Obstetrics &amp; Gynaecology Registrar (Accredited)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>General Medicine</t>
+          <t>Obstetrics</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Senior Registrar</t>
+          <t>Registrar</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Royal Children's Hospital</t>
+          <t>Grampians Health</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -8810,7 +9244,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
+          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Obstetrics-&amp;-Gynaecology-Registrar-%28Accredited%29-VIC-3350/1362508966/</t>
         </is>
       </c>
       <c r="K19" t="n">
@@ -8896,28 +9330,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Michael O'Brien</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Monash_Health</t>
+          <t>RCH</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2027 Diabetes &amp; Endocrinology Registrar - unaccredited</t>
+          <t>Neurology Consultant</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Consultant</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Monash Health</t>
+          <t>Royal Children's Hospital</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -8932,11 +9366,11 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://careers.monashhealth.org/job/Clayton-2027-Diabetes-&amp;-Endocrinology-Registrar-unaccredited-VIC-3168/1361886666/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Neurology-Consultant/1362944566/</t>
         </is>
       </c>
       <c r="K21" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -11345,7 +11779,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -11379,7 +11812,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -11417,7 +11849,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -11451,8 +11882,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -11485,7 +11914,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -11519,8 +11947,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -11533,7 +11959,6 @@
           <t>Psychiatry</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>Western Health</t>
@@ -11549,7 +11974,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -11583,8 +12007,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -12122,7 +12544,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -12156,8 +12577,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -12170,7 +12589,6 @@
           <t>ICU</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>Grampians Health</t>
@@ -12186,7 +12604,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -12220,8 +12637,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -12254,7 +12669,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -12288,8 +12702,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -12302,7 +12714,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>Grampians Health</t>
@@ -12318,7 +12729,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -12352,8 +12762,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -12386,7 +12794,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -12420,8 +12827,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -12429,7 +12834,6 @@
           <t>International Job Seekers</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>Intern</t>
@@ -12450,7 +12854,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -12484,8 +12887,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -13118,7 +13519,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>Eastern Health</t>
@@ -13134,7 +13534,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -13168,8 +13567,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -13177,7 +13574,6 @@
           <t>2027 Upper Gastro Intestinal Research Fellow</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>Fellow</t>
@@ -13198,7 +13594,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -13232,8 +13627,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -13288,11 +13681,11 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. Michael O'Brien</t>
         </is>
       </c>
       <c r="M63" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -13472,7 +13865,7 @@
         </is>
       </c>
       <c r="M66" t="n">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
@@ -13597,7 +13990,7 @@
         </is>
       </c>
       <c r="M68" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -13657,7 +14050,7 @@
         </is>
       </c>
       <c r="M69" t="n">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -14851,7 +15244,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -14885,7 +15277,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -14923,7 +15314,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -14957,7 +15347,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -14995,7 +15384,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15029,7 +15417,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -15067,7 +15454,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15101,7 +15487,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -15119,7 +15504,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -15135,7 +15519,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15169,8 +15552,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O95" t="inlineStr"/>
-      <c r="P95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -15183,7 +15564,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -15199,7 +15579,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15233,8 +15612,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O96" t="inlineStr"/>
-      <c r="P96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -15247,7 +15624,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -15263,7 +15639,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15297,8 +15672,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O97" t="inlineStr"/>
-      <c r="P97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -15311,7 +15684,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -15327,7 +15699,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15361,8 +15732,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O98" t="inlineStr"/>
-      <c r="P98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -15375,7 +15744,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -15391,7 +15759,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15425,8 +15792,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O99" t="inlineStr"/>
-      <c r="P99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -15439,7 +15804,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -15455,7 +15819,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15489,8 +15852,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O100" t="inlineStr"/>
-      <c r="P100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -15523,7 +15884,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15557,8 +15917,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O101" t="inlineStr"/>
-      <c r="P101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -15591,7 +15949,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15625,8 +15982,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O102" t="inlineStr"/>
-      <c r="P102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -15659,7 +16014,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15693,8 +16047,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O103" t="inlineStr"/>
-      <c r="P103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -15727,7 +16079,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
       <c r="H104" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15761,8 +16112,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O104" t="inlineStr"/>
-      <c r="P104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -15795,7 +16144,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15829,8 +16177,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O105" t="inlineStr"/>
-      <c r="P105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -15863,7 +16209,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15897,8 +16242,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O106" t="inlineStr"/>
-      <c r="P106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -15931,7 +16274,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -15965,8 +16307,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O107" t="inlineStr"/>
-      <c r="P107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -15979,7 +16319,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -15995,7 +16334,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
       <c r="H108" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -16029,8 +16367,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O108" t="inlineStr"/>
-      <c r="P108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -16038,7 +16374,6 @@
           <t>International Grants</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr">
         <is>
           <t>Intern</t>
@@ -16059,7 +16394,6 @@
           <t>NT</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -16093,8 +16427,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O109" t="inlineStr"/>
-      <c r="P109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -16102,7 +16434,6 @@
           <t>Prizes, grants, scholarships and fellowships</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
           <t>Fellow</t>
@@ -16123,7 +16454,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -16157,8 +16487,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O110" t="inlineStr"/>
-      <c r="P110" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19328,11 +19656,11 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. Michael O'Brien</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="H63" t="n">
         <v>30</v>
@@ -19482,7 +19810,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="H66" t="n">
         <v>30</v>
@@ -19582,7 +19910,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H68" t="n">
         <v>30</v>
@@ -19632,7 +19960,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="H69" t="n">
         <v>20</v>
@@ -24488,7 +24816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24496,7 +24824,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="47" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -24591,12 +24919,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Grampians_Health</t>
+          <t>RCH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Registrar - General Medicine Advanced Trainee</t>
+          <t>2027 Senior Registrar General Medicine</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -24606,12 +24934,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Senior Registrar</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Grampians Health</t>
+          <t>Royal Children's Hospital</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -24626,11 +24954,11 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Registrar-General-Medicine-Advanced-Trainee-VIC-3350/1362283766/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -24661,17 +24989,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Fractional Staff Specialist - Endocrinology</t>
+          <t>Registrar - General Medicine Advanced Trainee</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Endocrinology</t>
+          <t>General Medicine</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Registrar</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -24691,15 +25019,15 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Fractional-Staff-Specialist-Endocrinology-VIC-3350/1362736566/</t>
+          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Registrar-General-Medicine-Advanced-Trainee-VIC-3350/1362283766/</t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>63</v>
+        <v>88</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Good Match</t>
+          <t>High Match</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -24721,12 +25049,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Monash_Health</t>
+          <t>RCH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Consultant Paediatrician - Internal Locum</t>
+          <t>Neurology Consultant</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -24737,7 +25065,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Monash Health</t>
+          <t>Royal Children's Hospital</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -24752,15 +25080,15 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://careers.monashhealth.org/job/Clayton-Consultant-Paediatrician-Internal-Locum-VIC-3168/1363118266/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Neurology-Consultant/1362944566/</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Partial Match</t>
+          <t>Good Match</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -24782,15 +25110,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>RCH</t>
+          <t>Grampians_Health</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Neurology Consultant</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Fractional Staff Specialist - Endocrinology</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Endocrinology</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Consultant</t>
@@ -24798,7 +25130,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Royal Children's Hospital</t>
+          <t>Grampians Health</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -24813,15 +25145,15 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Neurology-Consultant/1362944566/</t>
+          <t>https://careers.grampianshealth.com/job/Ballarat-Central-Fractional-Staff-Specialist-Endocrinology-VIC-3350/1362736566/</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Partial Match</t>
+          <t>Good Match</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -24843,12 +25175,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Grampians_Health</t>
+          <t>Monash_Health</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Stawell - Consultant Anaesthetist</t>
+          <t>Consultant Paediatrician - Internal Locum</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -24859,7 +25191,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Grampians Health</t>
+          <t>Monash Health</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -24874,11 +25206,11 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://careers.grampianshealth.com/job/Stawell-Stawell-Consultant-Anaesthetist-VIC-3380/1363307366/</t>
+          <t>https://careers.monashhealth.org/job/Clayton-Consultant-Paediatrician-Internal-Locum-VIC-3168/1363118266/</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -24909,13 +25241,13 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>International Job Seekers</t>
+          <t>Stawell - Consultant Anaesthetist</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>Consultant</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -24935,15 +25267,15 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://www.gh.org.au/careers-and-training/international-recruitment/</t>
+          <t>https://careers.grampianshealth.com/job/Stawell-Stawell-Consultant-Anaesthetist-VIC-3380/1363307366/</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Low Match</t>
+          <t>Partial Match</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -24965,12 +25297,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>RACP</t>
+          <t>Grampians_Health</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>International Grants</t>
+          <t>International Job Seekers</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -24981,22 +25313,22 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>RACP Member Hospital (AU)</t>
+          <t>Grampians Health</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>nt</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/foundation/international-grants</t>
+          <t>https://www.gh.org.au/careers-and-training/international-recruitment/</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -25014,6 +25346,67 @@
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dr. Michael O'Brien</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>RACP</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>International Grants</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>RACP Member Hospital (AU)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>nt</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>NT</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://www.racp.edu.au/foundation/international-grants</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>28</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Low Match</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Yet to apply</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25026,22 +25419,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
@@ -25117,71 +25510,6 @@
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Dr. Sarah Williams</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>RCH</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2027 Senior Registrar General Medicine</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>General Medicine</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Senior Registrar</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Royal Children's Hospital</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>69</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Good Match</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Yet to apply</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -27446,7 +27774,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -27480,7 +27807,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
           <t>High Match</t>
@@ -27518,7 +27844,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -27552,8 +27877,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -27586,7 +27909,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -27620,8 +27942,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -27634,7 +27954,6 @@
           <t>Psychiatry</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Western Health</t>
@@ -27650,7 +27969,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>29-06-2026</t>
@@ -27684,8 +28002,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Doctor jobs update - 02 Jul 2026 14:00 AEST
</commit_message>
<xml_diff>
--- a/Job_Tracker.xlsx
+++ b/Job_Tracker.xlsx
@@ -1878,7 +1878,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>02-07-2026</t>
@@ -1927,7 +1926,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr">
         <is>
           <t>Weak title relevance; Specialty mismatch</t>
@@ -1945,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S12"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1964,7 +1962,7 @@
     <col width="24" customWidth="1" min="14" max="14"/>
     <col width="29" customWidth="1" min="15" max="15"/>
     <col width="55" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="55" customWidth="1" min="19" max="19"/>
   </cols>
@@ -2957,6 +2955,89 @@
         </is>
       </c>
       <c r="S12" t="inlineStr">
+        <is>
+          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Palliative Medicine - Internal Locum</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Eastern Health</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>02-07-2026 14:00</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://careers.easternhealth.org.au/job/Burwood-East-Palliative-Medicine-Internal-Locum-VIC-3151/1363692566/</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Eastern_Health</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Dr. Ananya Patel</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>21</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>static_html</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Primary — configured method</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Yet to apply</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
         <is>
           <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
         </is>
@@ -6293,7 +6374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11089,6 +11170,534 @@
         <v>0</v>
       </c>
       <c r="G145" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>SmartJobs_QLD</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Jobs_NT</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>0</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Careers_VIC</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" t="n">
+        <v>3</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Monash_Health</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" t="n">
+        <v>24</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Western_Health</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>static_html</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" t="n">
+        <v>18</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>WA_Health</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" t="n">
+        <v>25</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Peninsula_Health</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>The_Womens</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>playwright</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" t="n">
+        <v>1</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Grampians_Health</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>static_html</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" t="n">
+        <v>15</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Eastern_Health</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>static_html</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>1</v>
+      </c>
+      <c r="F155" t="n">
+        <v>12</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>RCH</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>static_html</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" t="n">
+        <v>8</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>RANZCOG</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>RACP</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>static_html</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" t="n">
+        <v>24</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>JobRadars</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>PageUp</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>all_methods_failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>02-07-2026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Mercy_Workday</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="inlineStr">
         <is>
           <t>all_methods_failed</t>
         </is>
@@ -13215,7 +13824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S130"/>
+  <dimension ref="A1:S131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -19043,7 +19652,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr">
         <is>
           <t>02-07-2026</t>
@@ -19092,7 +19700,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="R71" t="inlineStr"/>
       <c r="S71" t="inlineStr">
         <is>
           <t>Weak title relevance; Specialty mismatch; Location mismatch</t>
@@ -20362,7 +20969,6 @@
           <t>VIC</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
           <t>02-07-2026</t>
@@ -20411,7 +21017,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="R87" t="inlineStr"/>
       <c r="S87" t="inlineStr">
         <is>
           <t>Weak title relevance; Specialty mismatch</t>
@@ -21317,22 +21922,18 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2027 Senior Registrar General Medicine</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Internal Medicine</t>
-        </is>
-      </c>
+          <t>Palliative Medicine - Internal Locum</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Senior Registrar</t>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Royal Children's Hospital</t>
+          <t>Eastern Health</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -21345,33 +21946,34 @@
           <t>VIC</t>
         </is>
       </c>
+      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>02-07-2026</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>30-06-2026 21:27</t>
+          <t>02-07-2026 14:00</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
+          <t>https://careers.easternhealth.org.au/job/Burwood-East-Palliative-Medicine-Internal-Locum-VIC-3151/1363692566/</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>RCH</t>
+          <t>Eastern_Health</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="M99" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -21385,29 +21987,35 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>Weak title relevance; Experience level mismatch</t>
+          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>2 days old</t>
-        </is>
-      </c>
+          <t>Yet to apply</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr"/>
       <c r="S99" t="inlineStr">
         <is>
-          <t>Weak title relevance; Experience level mismatch</t>
+          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2027 Paediatric Registrars VPAT (Advanced and Continuing Trainees)</t>
+          <t>2027 Senior Registrar General Medicine</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Senior Registrar</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -21437,7 +22045,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Paediatric-Registrars-VPAT-%28Advanced-and-Continuing-Trainees%29/1361643566/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -21447,11 +22055,11 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="M100" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -21465,7 +22073,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>Weak title relevance; Specialty mismatch</t>
+          <t>Weak title relevance; Experience level mismatch</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -21475,19 +22083,14 @@
       </c>
       <c r="S100" t="inlineStr">
         <is>
-          <t>Weak title relevance; Specialty mismatch</t>
+          <t>Weak title relevance; Experience level mismatch</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2027 Immunopathology Registrar / Fellow</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Pathology</t>
+          <t>2027 Paediatric Registrars VPAT (Advanced and Continuing Trainees)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -21522,7 +22125,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Immunopathology-Registrar-Fellow/1363389666/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Paediatric-Registrars-VPAT-%28Advanced-and-Continuing-Trainees%29/1361643566/</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -21532,11 +22135,11 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>Dr. Priya Sharma</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="M101" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -21567,12 +22170,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2027 RCH NICU - VPAT Registrar</t>
+          <t>2027 Immunopathology Registrar / Fellow</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ICU</t>
+          <t>Pathology</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -21607,7 +22210,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-RCH-NICU-VPAT-Registrar/1363270566/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Immunopathology-Registrar-Fellow/1363389666/</t>
         </is>
       </c>
       <c r="K102" t="inlineStr">
@@ -21617,11 +22220,11 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Priya Sharma</t>
         </is>
       </c>
       <c r="M102" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -21652,7 +22255,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Microbiology Registrar 2027</t>
+          <t>2027 RCH NICU - VPAT Registrar</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ICU</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -21687,7 +22295,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Microbiology-Registrar-2027/1363255766/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-RCH-NICU-VPAT-Registrar/1363270566/</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
@@ -21732,7 +22340,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2027 Allergy &amp; Immunology Fellow / Registrar</t>
+          <t>Microbiology Registrar 2027</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -21767,7 +22375,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Allergy-&amp;-Immunology-Fellow-Registrar/1363326766/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Microbiology-Registrar-2027/1363255766/</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -21781,7 +22389,7 @@
         </is>
       </c>
       <c r="M104" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -21812,17 +22420,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Neurology Consultant</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Neurology</t>
+          <t>2027 Allergy &amp; Immunology Fellow / Registrar</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Consultant</t>
+          <t>Registrar</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -21852,7 +22455,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Neurology-Consultant/1362944566/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Allergy-&amp;-Immunology-Fellow-Registrar/1363326766/</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -21862,11 +22465,11 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>Dr. Michael O'Brien</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="M105" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -21897,17 +22500,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2027 Unaccredited Ophthalmology Registrar</t>
+          <t>Neurology Consultant</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Ophthalmology</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Registrar</t>
+          <t>Consultant</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -21927,17 +22530,17 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>01-07-2026</t>
+          <t>30-06-2026</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>01-07-2026 09:20</t>
+          <t>30-06-2026 21:27</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Unaccredited-Ophthalmology-Registrar/1357689666/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Neurology-Consultant/1362944566/</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -21947,11 +22550,11 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Michael O'Brien</t>
         </is>
       </c>
       <c r="M106" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -21970,7 +22573,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>1 day old</t>
+          <t>2 days old</t>
         </is>
       </c>
       <c r="S106" t="inlineStr">
@@ -21982,61 +22585,61 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Paediatrics &amp; Child Health</t>
+          <t>2027 Unaccredited Ophthalmology Registrar</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Internal Medicine</t>
+          <t>Ophthalmology</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Fellow</t>
+          <t>Registrar</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>RACP Member Hospital (AU)</t>
+          <t>Royal Children's Hospital</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>nt</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>01-07-2026</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>30-06-2026 21:27</t>
+          <t>01-07-2026 09:20</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/basic-training/paediatrics-child-health</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Unaccredited-Ophthalmology-Registrar/1357689666/</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>RACP</t>
+          <t>RCH</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="M107" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
@@ -22050,24 +22653,24 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>Weak title relevance; Experience level mismatch</t>
+          <t>Weak title relevance; Specialty mismatch</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>2 days old</t>
+          <t>1 day old</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
         <is>
-          <t>Weak title relevance; Experience level mismatch</t>
+          <t>Weak title relevance; Specialty mismatch</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Adult Internal Medicine</t>
+          <t>Paediatrics &amp; Child Health</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -22107,7 +22710,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/basic-training/adult-internal-medicine</t>
+          <t>https://www.racp.edu.au/trainees/basic-training/paediatrics-child-health</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -22121,7 +22724,7 @@
         </is>
       </c>
       <c r="M108" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -22152,7 +22755,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Adolescent and Young Adult Medicine</t>
+          <t>Adult Internal Medicine</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -22192,7 +22795,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/adolescent-and-young-adult-medicine</t>
+          <t>https://www.racp.edu.au/trainees/basic-training/adult-internal-medicine</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -22237,7 +22840,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Addiction Medicine</t>
+          <t>Adolescent and Young Adult Medicine</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -22277,7 +22880,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/addiction-medicine</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/adolescent-and-young-adult-medicine</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -22291,7 +22894,7 @@
         </is>
       </c>
       <c r="M110" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -22322,7 +22925,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>New curricula</t>
+          <t>Addiction Medicine</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -22362,7 +22965,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/new-curricula</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/addiction-medicine</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -22407,7 +23010,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Advanced Training - New Curricula</t>
+          <t>New curricula</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -22447,7 +23050,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/recognition-of-prior-learning/advanced-training-new-curricula</t>
+          <t>https://www.racp.edu.au/trainees/new-curricula</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -22461,7 +23064,7 @@
         </is>
       </c>
       <c r="M112" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -22492,7 +23095,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Advanced Training - New Curricula</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -22532,7 +23135,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/cardiology</t>
+          <t>https://www.racp.edu.au/trainees/recognition-of-prior-learning/advanced-training-new-curricula</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -22546,7 +23149,7 @@
         </is>
       </c>
       <c r="M113" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -22577,7 +23180,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Post-Fellowship training</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -22617,7 +23220,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/multi-specialty-training-options/post-fellowship-training</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/cardiology</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -22631,7 +23234,7 @@
         </is>
       </c>
       <c r="M114" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
@@ -22662,7 +23265,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Prizes, grants, scholarships and fellowships</t>
+          <t>Post-Fellowship training</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -22697,7 +23305,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/become-a-physician/prizes-grants-scholarships-and-fellowships</t>
+          <t>https://www.racp.edu.au/trainees/multi-specialty-training-options/post-fellowship-training</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -22711,7 +23319,7 @@
         </is>
       </c>
       <c r="M115" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -22725,7 +23333,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
+          <t>Weak title relevance; Experience level mismatch</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
@@ -22735,19 +23343,19 @@
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
+          <t>Weak title relevance; Experience level mismatch</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>The President's Message</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>ENT</t>
+          <t>Prizes, grants, scholarships and fellowships</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Fellow</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -22762,7 +23370,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -22777,7 +23385,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/news-and-events/presidents-message</t>
+          <t>https://www.racp.edu.au/become-a-physician/prizes-grants-scholarships-and-fellowships</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -22791,7 +23399,7 @@
         </is>
       </c>
       <c r="M116" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -22822,7 +23430,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Supervisor Professional Development Program</t>
+          <t>The President's Message</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -22830,11 +23438,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Fellow</t>
-        </is>
-      </c>
       <c r="D117" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -22862,7 +23465,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/supervision/supervisor-professional-development-program</t>
+          <t>https://www.racp.edu.au/news-and-events/presidents-message</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -22872,7 +23475,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="M117" t="n">
@@ -22907,7 +23510,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Represent your Profession</t>
+          <t>Supervisor Professional Development Program</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -22915,6 +23518,11 @@
           <t>ENT</t>
         </is>
       </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Fellow</t>
+        </is>
+      </c>
       <c r="D118" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -22942,7 +23550,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/policy-and-advocacy/represent-your-profession</t>
+          <t>https://www.racp.edu.au/fellows/supervision/supervisor-professional-development-program</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -22952,7 +23560,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="M118" t="n">
@@ -22987,7 +23595,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Continuing Professional Development</t>
+          <t>Represent your Profession</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -22995,11 +23603,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Fellow</t>
-        </is>
-      </c>
       <c r="D119" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -23027,7 +23630,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/continuing-professional-development</t>
+          <t>https://www.racp.edu.au/policy-and-advocacy/represent-your-profession</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -23037,11 +23640,11 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="M119" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -23072,7 +23675,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CPD Recognition and Assessment Framework</t>
+          <t>Continuing Professional Development</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -23112,7 +23715,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework</t>
+          <t>https://www.racp.edu.au/fellows/continuing-professional-development</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -23157,7 +23760,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CAPE Program-Level Requirements</t>
+          <t>CPD Recognition and Assessment Framework</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -23197,7 +23800,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework/cape-program-level-requirements</t>
+          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -23207,7 +23810,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="M121" t="n">
@@ -23242,7 +23845,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Prevocational Training and Entry to Basic Training</t>
+          <t>CAPE Program-Level Requirements</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -23250,6 +23853,11 @@
           <t>ENT</t>
         </is>
       </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Fellow</t>
+        </is>
+      </c>
       <c r="D122" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -23277,7 +23885,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/become-a-physician/entry-into-basic-training/prevocational-training-and-entry-to-basic-training</t>
+          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework/cape-program-level-requirements</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -23291,7 +23899,7 @@
         </is>
       </c>
       <c r="M122" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
@@ -23322,7 +23930,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Position design and posting</t>
+          <t>Prevocational Training and Entry to Basic Training</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -23330,11 +23938,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Fellow</t>
-        </is>
-      </c>
       <c r="D123" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -23362,7 +23965,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/local-selection/position-design-and-posting</t>
+          <t>https://www.racp.edu.au/become-a-physician/entry-into-basic-training/prevocational-training-and-entry-to-basic-training</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -23407,7 +24010,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Student Scholarships &amp; Prizes</t>
+          <t>Position design and posting</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -23415,6 +24018,11 @@
           <t>ENT</t>
         </is>
       </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Fellow</t>
+        </is>
+      </c>
       <c r="D124" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -23442,7 +24050,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/foundation/student-scholarships-and-prizes</t>
+          <t>https://www.racp.edu.au/fellows/local-selection/position-design-and-posting</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -23452,11 +24060,11 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="M124" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N124" t="inlineStr">
         <is>
@@ -23487,7 +24095,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Selection into Training Quality Assurance and Improvement</t>
+          <t>Student Scholarships &amp; Prizes</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -23522,7 +24130,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/become-a-physician/selection-into-training-quality-assurance-and-improvement</t>
+          <t>https://www.racp.edu.au/foundation/student-scholarships-and-prizes</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -23567,7 +24175,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Becoming a Fellow</t>
+          <t>Selection into Training Quality Assurance and Improvement</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -23575,11 +24183,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Fellow</t>
-        </is>
-      </c>
       <c r="D126" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -23607,7 +24210,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/becoming-a-fellow</t>
+          <t>https://www.racp.edu.au/become-a-physician/selection-into-training-quality-assurance-and-improvement</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -23617,7 +24220,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="M126" t="n">
@@ -23652,12 +24255,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>International Grants</t>
+          <t>Becoming a Fellow</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>ENT</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>Fellow</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -23687,7 +24295,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/foundation/international-grants</t>
+          <t>https://www.racp.edu.au/fellows/becoming-a-fellow</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -23701,7 +24309,7 @@
         </is>
       </c>
       <c r="M127" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
@@ -23732,12 +24340,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Our recipients</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>ENT</t>
+          <t>International Grants</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Intern</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -23767,7 +24375,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/foundation/our-recipients</t>
+          <t>https://www.racp.edu.au/foundation/international-grants</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -23812,7 +24420,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>News &amp; Events</t>
+          <t>Our recipients</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -23847,7 +24455,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/news-and-events</t>
+          <t>https://www.racp.edu.au/foundation/our-recipients</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -23857,11 +24465,11 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="M129" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -23892,7 +24500,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>New Fellow Survey</t>
+          <t>News &amp; Events</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -23900,11 +24508,6 @@
           <t>ENT</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Fellow</t>
-        </is>
-      </c>
       <c r="D130" t="inlineStr">
         <is>
           <t>RACP Member Hospital (AU)</t>
@@ -23932,7 +24535,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/becoming-a-fellow/new-fellow-survey</t>
+          <t>https://www.racp.edu.au/news-and-events</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -23942,7 +24545,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="M130" t="n">
@@ -23969,6 +24572,91 @@
         </is>
       </c>
       <c r="S130" t="inlineStr">
+        <is>
+          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>New Fellow Survey</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>ENT</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Fellow</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>RACP Member Hospital (AU)</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>nt</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>NT</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>30-06-2026 21:27</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://www.racp.edu.au/fellows/becoming-a-fellow/new-fellow-survey</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>RACP</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Dr. James Chen</t>
+        </is>
+      </c>
+      <c r="M131" t="n">
+        <v>12</v>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>static_html</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>Primary — configured method</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
+        </is>
+      </c>
+      <c r="Q131" t="inlineStr">
+        <is>
+          <t>2 days old</t>
+        </is>
+      </c>
+      <c r="S131" t="inlineStr">
         <is>
           <t>Weak title relevance; Specialty mismatch; Experience level mismatch</t>
         </is>
@@ -23985,7 +24673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -28917,17 +29605,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2027 Senior Registrar General Medicine</t>
+          <t>Palliative Medicine - Internal Locum</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>RCH</t>
+          <t>Eastern_Health</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Royal Children's Hospital</t>
+          <t>Eastern Health</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -28937,37 +29625,37 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
+          <t>https://careers.easternhealth.org.au/job/Burwood-East-Palliative-Medicine-Internal-Locum-VIC-3151/1363692566/</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="H99" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="I99" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="J99" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="K99" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="L99" t="n">
-        <v>42</v>
+        <v>18</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2027 Paediatric Registrars VPAT (Advanced and Continuing Trainees)</t>
+          <t>2027 Senior Registrar General Medicine</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -28987,37 +29675,37 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Paediatric-Registrars-VPAT-%28Advanced-and-Continuing-Trainees%29/1361643566/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Senior-Registrar-General-Medicine/1362878366/</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="G100" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H100" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I100" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="J100" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K100" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="L100" t="n">
-        <v>11</v>
+        <v>42</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2027 Immunopathology Registrar / Fellow</t>
+          <t>2027 Paediatric Registrars VPAT (Advanced and Continuing Trainees)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -29037,37 +29725,37 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Immunopathology-Registrar-Fellow/1363389666/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Paediatric-Registrars-VPAT-%28Advanced-and-Continuing-Trainees%29/1361643566/</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Dr. Priya Sharma</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="G101" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H101" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="I101" t="n">
         <v>16</v>
       </c>
       <c r="J101" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="K101" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="L101" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2027 RCH NICU - VPAT Registrar</t>
+          <t>2027 Immunopathology Registrar / Fellow</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -29087,37 +29775,37 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-RCH-NICU-VPAT-Registrar/1363270566/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Immunopathology-Registrar-Fellow/1363389666/</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Priya Sharma</t>
         </is>
       </c>
       <c r="G102" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H102" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="I102" t="n">
+        <v>16</v>
+      </c>
+      <c r="J102" t="n">
+        <v>35</v>
+      </c>
+      <c r="K102" t="n">
         <v>12</v>
       </c>
-      <c r="J102" t="n">
-        <v>34</v>
-      </c>
-      <c r="K102" t="n">
-        <v>13</v>
-      </c>
       <c r="L102" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Microbiology Registrar 2027</t>
+          <t>2027 RCH NICU - VPAT Registrar</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -29137,7 +29825,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Microbiology-Registrar-2027/1363255766/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-RCH-NICU-VPAT-Registrar/1363270566/</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -29149,10 +29837,10 @@
         <v>34</v>
       </c>
       <c r="H103" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I103" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J103" t="n">
         <v>34</v>
@@ -29161,13 +29849,13 @@
         <v>13</v>
       </c>
       <c r="L103" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2027 Allergy &amp; Immunology Fellow / Registrar</t>
+          <t>Microbiology Registrar 2027</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -29187,7 +29875,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Allergy-&amp;-Immunology-Fellow-Registrar/1363326766/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Microbiology-Registrar-2027/1363255766/</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -29196,28 +29884,28 @@
         </is>
       </c>
       <c r="G104" t="n">
+        <v>34</v>
+      </c>
+      <c r="H104" t="n">
         <v>33</v>
-      </c>
-      <c r="H104" t="n">
-        <v>32</v>
       </c>
       <c r="I104" t="n">
         <v>15</v>
       </c>
       <c r="J104" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K104" t="n">
+        <v>13</v>
+      </c>
+      <c r="L104" t="n">
         <v>14</v>
-      </c>
-      <c r="L104" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Neurology Consultant</t>
+          <t>2027 Allergy &amp; Immunology Fellow / Registrar</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -29237,28 +29925,28 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Neurology-Consultant/1362944566/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Allergy-&amp;-Immunology-Fellow-Registrar/1363326766/</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Dr. Michael O'Brien</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="G105" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H105" t="n">
+        <v>32</v>
+      </c>
+      <c r="I105" t="n">
         <v>15</v>
       </c>
-      <c r="I105" t="n">
+      <c r="J105" t="n">
+        <v>33</v>
+      </c>
+      <c r="K105" t="n">
         <v>14</v>
-      </c>
-      <c r="J105" t="n">
-        <v>14</v>
-      </c>
-      <c r="K105" t="n">
-        <v>31</v>
       </c>
       <c r="L105" t="n">
         <v>12</v>
@@ -29267,7 +29955,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2027 Unaccredited Ophthalmology Registrar</t>
+          <t>Neurology Consultant</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -29287,87 +29975,87 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Unaccredited-Ophthalmology-Registrar/1357689666/</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-Neurology-Consultant/1362944566/</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Dr. Ananya Patel</t>
+          <t>Dr. Michael O'Brien</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H106" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="I106" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J106" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="K106" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="L106" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Paediatrics &amp; Child Health</t>
+          <t>2027 Unaccredited Ophthalmology Registrar</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>RACP</t>
+          <t>RCH</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>RACP Member Hospital (AU)</t>
+          <t>Royal Children's Hospital</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/basic-training/paediatrics-child-health</t>
+          <t>https://careers.rch.org.au/job/50-Flemington-Rd-2027-Unaccredited-Ophthalmology-Registrar/1357689666/</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Ananya Patel</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="H107" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="I107" t="n">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="J107" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="K107" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="L107" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Adult Internal Medicine</t>
+          <t>Paediatrics &amp; Child Health</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -29387,7 +30075,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/basic-training/adult-internal-medicine</t>
+          <t>https://www.racp.edu.au/trainees/basic-training/paediatrics-child-health</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -29396,19 +30084,19 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H108" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I108" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J108" t="n">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="K108" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="L108" t="n">
         <v>36</v>
@@ -29417,7 +30105,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Adolescent and Young Adult Medicine</t>
+          <t>Adult Internal Medicine</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -29437,7 +30125,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/adolescent-and-young-adult-medicine</t>
+          <t>https://www.racp.edu.au/trainees/basic-training/adult-internal-medicine</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -29449,25 +30137,25 @@
         <v>42</v>
       </c>
       <c r="H109" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I109" t="n">
         <v>42</v>
       </c>
       <c r="J109" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K109" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="L109" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Addiction Medicine</t>
+          <t>Adolescent and Young Adult Medicine</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -29487,7 +30175,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/addiction-medicine</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/adolescent-and-young-adult-medicine</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -29496,28 +30184,28 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H110" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I110" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J110" t="n">
         <v>11</v>
       </c>
       <c r="K110" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L110" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>New curricula</t>
+          <t>Addiction Medicine</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -29537,7 +30225,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/new-curricula</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/addiction-medicine</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -29549,25 +30237,25 @@
         <v>41</v>
       </c>
       <c r="H111" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I111" t="n">
         <v>41</v>
       </c>
       <c r="J111" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="K111" t="n">
         <v>34</v>
       </c>
       <c r="L111" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Advanced Training - New Curricula</t>
+          <t>New curricula</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -29587,7 +30275,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/recognition-of-prior-learning/advanced-training-new-curricula</t>
+          <t>https://www.racp.edu.au/trainees/new-curricula</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -29596,19 +30284,19 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H112" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I112" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J112" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K112" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="L112" t="n">
         <v>35</v>
@@ -29617,7 +30305,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Cardiology</t>
+          <t>Advanced Training - New Curricula</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -29637,7 +30325,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/advanced-training/cardiology</t>
+          <t>https://www.racp.edu.au/trainees/recognition-of-prior-learning/advanced-training-new-curricula</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -29646,28 +30334,28 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H113" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I113" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J113" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K113" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="L113" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Post-Fellowship training</t>
+          <t>Cardiology</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -29687,7 +30375,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/trainees/multi-specialty-training-options/post-fellowship-training</t>
+          <t>https://www.racp.edu.au/trainees/advanced-training/cardiology</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -29696,28 +30384,28 @@
         </is>
       </c>
       <c r="G114" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H114" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I114" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J114" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K114" t="n">
         <v>33</v>
       </c>
       <c r="L114" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Prizes, grants, scholarships and fellowships</t>
+          <t>Post-Fellowship training</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -29737,7 +30425,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/become-a-physician/prizes-grants-scholarships-and-fellowships</t>
+          <t>https://www.racp.edu.au/trainees/multi-specialty-training-options/post-fellowship-training</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -29746,28 +30434,28 @@
         </is>
       </c>
       <c r="G115" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="H115" t="n">
         <v>8</v>
       </c>
       <c r="I115" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="J115" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K115" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="L115" t="n">
-        <v>14</v>
+        <v>35</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>The President's Message</t>
+          <t>Prizes, grants, scholarships and fellowships</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -29782,12 +30470,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>NT</t>
+          <t>WA</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/news-and-events/presidents-message</t>
+          <t>https://www.racp.edu.au/become-a-physician/prizes-grants-scholarships-and-fellowships</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -29796,28 +30484,28 @@
         </is>
       </c>
       <c r="G116" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="H116" t="n">
+        <v>8</v>
+      </c>
+      <c r="I116" t="n">
+        <v>22</v>
+      </c>
+      <c r="J116" t="n">
         <v>9</v>
       </c>
-      <c r="I116" t="n">
-        <v>17</v>
-      </c>
-      <c r="J116" t="n">
-        <v>10</v>
-      </c>
       <c r="K116" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="L116" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Supervisor Professional Development Program</t>
+          <t>The President's Message</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -29837,12 +30525,12 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/supervision/supervisor-professional-development-program</t>
+          <t>https://www.racp.edu.au/news-and-events/presidents-message</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="G117" t="n">
@@ -29852,22 +30540,22 @@
         <v>9</v>
       </c>
       <c r="I117" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J117" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K117" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="L117" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Represent your Profession</t>
+          <t>Supervisor Professional Development Program</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -29887,37 +30575,37 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/policy-and-advocacy/represent-your-profession</t>
+          <t>https://www.racp.edu.au/fellows/supervision/supervisor-professional-development-program</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="G118" t="n">
         <v>17</v>
       </c>
       <c r="H118" t="n">
+        <v>9</v>
+      </c>
+      <c r="I118" t="n">
+        <v>16</v>
+      </c>
+      <c r="J118" t="n">
+        <v>9</v>
+      </c>
+      <c r="K118" t="n">
         <v>8</v>
       </c>
-      <c r="I118" t="n">
+      <c r="L118" t="n">
         <v>17</v>
-      </c>
-      <c r="J118" t="n">
-        <v>10</v>
-      </c>
-      <c r="K118" t="n">
-        <v>9</v>
-      </c>
-      <c r="L118" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Continuing Professional Development</t>
+          <t>Represent your Profession</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -29937,37 +30625,37 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/continuing-professional-development</t>
+          <t>https://www.racp.edu.au/policy-and-advocacy/represent-your-profession</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H119" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I119" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="J119" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K119" t="n">
         <v>9</v>
       </c>
       <c r="L119" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CPD Recognition and Assessment Framework</t>
+          <t>Continuing Professional Development</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -29987,7 +30675,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework</t>
+          <t>https://www.racp.edu.au/fellows/continuing-professional-development</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -29999,16 +30687,16 @@
         <v>16</v>
       </c>
       <c r="H120" t="n">
+        <v>6</v>
+      </c>
+      <c r="I120" t="n">
+        <v>14</v>
+      </c>
+      <c r="J120" t="n">
         <v>9</v>
       </c>
-      <c r="I120" t="n">
-        <v>15</v>
-      </c>
-      <c r="J120" t="n">
-        <v>10</v>
-      </c>
       <c r="K120" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L120" t="n">
         <v>16</v>
@@ -30017,7 +30705,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CAPE Program-Level Requirements</t>
+          <t>CPD Recognition and Assessment Framework</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -30037,37 +30725,37 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework/cape-program-level-requirements</t>
+          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="G121" t="n">
         <v>16</v>
       </c>
       <c r="H121" t="n">
+        <v>9</v>
+      </c>
+      <c r="I121" t="n">
+        <v>15</v>
+      </c>
+      <c r="J121" t="n">
+        <v>10</v>
+      </c>
+      <c r="K121" t="n">
         <v>8</v>
       </c>
-      <c r="I121" t="n">
+      <c r="L121" t="n">
         <v>16</v>
-      </c>
-      <c r="J121" t="n">
-        <v>6</v>
-      </c>
-      <c r="K121" t="n">
-        <v>5</v>
-      </c>
-      <c r="L121" t="n">
-        <v>15</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Prevocational Training and Entry to Basic Training</t>
+          <t>CAPE Program-Level Requirements</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -30087,7 +30775,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/become-a-physician/entry-into-basic-training/prevocational-training-and-entry-to-basic-training</t>
+          <t>https://www.racp.edu.au/fellows/cpd-recognition-assessment-framework/cape-program-level-requirements</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -30096,28 +30784,28 @@
         </is>
       </c>
       <c r="G122" t="n">
+        <v>16</v>
+      </c>
+      <c r="H122" t="n">
+        <v>8</v>
+      </c>
+      <c r="I122" t="n">
+        <v>16</v>
+      </c>
+      <c r="J122" t="n">
+        <v>6</v>
+      </c>
+      <c r="K122" t="n">
+        <v>5</v>
+      </c>
+      <c r="L122" t="n">
         <v>15</v>
-      </c>
-      <c r="H122" t="n">
-        <v>10</v>
-      </c>
-      <c r="I122" t="n">
-        <v>15</v>
-      </c>
-      <c r="J122" t="n">
-        <v>8</v>
-      </c>
-      <c r="K122" t="n">
-        <v>11</v>
-      </c>
-      <c r="L122" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Position design and posting</t>
+          <t>Prevocational Training and Entry to Basic Training</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -30137,7 +30825,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/local-selection/position-design-and-posting</t>
+          <t>https://www.racp.edu.au/become-a-physician/entry-into-basic-training/prevocational-training-and-entry-to-basic-training</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -30149,7 +30837,7 @@
         <v>15</v>
       </c>
       <c r="H123" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I123" t="n">
         <v>15</v>
@@ -30158,16 +30846,16 @@
         <v>8</v>
       </c>
       <c r="K123" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="L123" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Student Scholarships &amp; Prizes</t>
+          <t>Position design and posting</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -30187,37 +30875,37 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/foundation/student-scholarships-and-prizes</t>
+          <t>https://www.racp.edu.au/fellows/local-selection/position-design-and-posting</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="G124" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H124" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I124" t="n">
+        <v>15</v>
+      </c>
+      <c r="J124" t="n">
+        <v>8</v>
+      </c>
+      <c r="K124" t="n">
+        <v>5</v>
+      </c>
+      <c r="L124" t="n">
         <v>13</v>
-      </c>
-      <c r="J124" t="n">
-        <v>7</v>
-      </c>
-      <c r="K124" t="n">
-        <v>8</v>
-      </c>
-      <c r="L124" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Selection into Training Quality Assurance and Improvement</t>
+          <t>Student Scholarships &amp; Prizes</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -30237,7 +30925,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/become-a-physician/selection-into-training-quality-assurance-and-improvement</t>
+          <t>https://www.racp.edu.au/foundation/student-scholarships-and-prizes</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -30249,16 +30937,16 @@
         <v>14</v>
       </c>
       <c r="H125" t="n">
+        <v>10</v>
+      </c>
+      <c r="I125" t="n">
+        <v>13</v>
+      </c>
+      <c r="J125" t="n">
+        <v>7</v>
+      </c>
+      <c r="K125" t="n">
         <v>8</v>
-      </c>
-      <c r="I125" t="n">
-        <v>9</v>
-      </c>
-      <c r="J125" t="n">
-        <v>9</v>
-      </c>
-      <c r="K125" t="n">
-        <v>10</v>
       </c>
       <c r="L125" t="n">
         <v>14</v>
@@ -30267,7 +30955,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Becoming a Fellow</t>
+          <t>Selection into Training Quality Assurance and Improvement</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -30287,12 +30975,12 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/becoming-a-fellow</t>
+          <t>https://www.racp.edu.au/become-a-physician/selection-into-training-quality-assurance-and-improvement</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="G126" t="n">
@@ -30302,22 +30990,22 @@
         <v>8</v>
       </c>
       <c r="I126" t="n">
+        <v>9</v>
+      </c>
+      <c r="J126" t="n">
+        <v>9</v>
+      </c>
+      <c r="K126" t="n">
+        <v>10</v>
+      </c>
+      <c r="L126" t="n">
         <v>14</v>
-      </c>
-      <c r="J126" t="n">
-        <v>6</v>
-      </c>
-      <c r="K126" t="n">
-        <v>3</v>
-      </c>
-      <c r="L126" t="n">
-        <v>13</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>International Grants</t>
+          <t>Becoming a Fellow</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -30337,7 +31025,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/foundation/international-grants</t>
+          <t>https://www.racp.edu.au/fellows/becoming-a-fellow</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -30346,19 +31034,19 @@
         </is>
       </c>
       <c r="G127" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H127" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I127" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J127" t="n">
         <v>6</v>
       </c>
       <c r="K127" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L127" t="n">
         <v>13</v>
@@ -30367,7 +31055,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Our recipients</t>
+          <t>International Grants</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -30387,7 +31075,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/foundation/our-recipients</t>
+          <t>https://www.racp.edu.au/foundation/international-grants</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -30399,25 +31087,25 @@
         <v>13</v>
       </c>
       <c r="H128" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I128" t="n">
         <v>13</v>
       </c>
       <c r="J128" t="n">
+        <v>6</v>
+      </c>
+      <c r="K128" t="n">
         <v>7</v>
       </c>
-      <c r="K128" t="n">
-        <v>6</v>
-      </c>
       <c r="L128" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>News &amp; Events</t>
+          <t>Our recipients</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -30437,25 +31125,25 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/news-and-events</t>
+          <t>https://www.racp.edu.au/foundation/our-recipients</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Dr. Sarah Williams</t>
+          <t>Dr. James Chen</t>
         </is>
       </c>
       <c r="G129" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H129" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I129" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J129" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K129" t="n">
         <v>6</v>
@@ -30467,7 +31155,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>New Fellow Survey</t>
+          <t>News &amp; Events</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -30487,30 +31175,80 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://www.racp.edu.au/fellows/becoming-a-fellow/new-fellow-survey</t>
+          <t>https://www.racp.edu.au/news-and-events</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Dr. James Chen</t>
+          <t>Dr. Sarah Williams</t>
         </is>
       </c>
       <c r="G130" t="n">
         <v>12</v>
       </c>
       <c r="H130" t="n">
+        <v>5</v>
+      </c>
+      <c r="I130" t="n">
+        <v>11</v>
+      </c>
+      <c r="J130" t="n">
         <v>6</v>
-      </c>
-      <c r="I130" t="n">
-        <v>12</v>
-      </c>
-      <c r="J130" t="n">
-        <v>5</v>
       </c>
       <c r="K130" t="n">
         <v>6</v>
       </c>
       <c r="L130" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>New Fellow Survey</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>RACP</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>RACP Member Hospital (AU)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>NT</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>https://www.racp.edu.au/fellows/becoming-a-fellow/new-fellow-survey</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Dr. James Chen</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>12</v>
+      </c>
+      <c r="H131" t="n">
+        <v>6</v>
+      </c>
+      <c r="I131" t="n">
+        <v>12</v>
+      </c>
+      <c r="J131" t="n">
+        <v>5</v>
+      </c>
+      <c r="K131" t="n">
+        <v>6</v>
+      </c>
+      <c r="L131" t="n">
         <v>12</v>
       </c>
     </row>
@@ -42779,7 +43517,6 @@
           <t>WA</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>02-07-2026</t>
@@ -42828,7 +43565,6 @@
           <t>Yet to apply</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr">
         <is>
           <t>Weak title relevance; Specialty mismatch; Location mismatch</t>

</xml_diff>